<commit_message>
feat: implement comprehensive reward analysis pipeline and auxiliary reward handlers for CartPole simulations.
</commit_message>
<xml_diff>
--- a/0_bkp/Planning Simulations.xlsx
+++ b/0_bkp/Planning Simulations.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\davor\Escritorio\DOCTORADO\Tesis\RL_5_SimpleSystemSimulator\0_bkp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A61099E-9C62-4538-9532-B2AE15F16A20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01DFF6CC-ABF3-4EF9-9C02-4BB71321524F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{ADA15B25-271F-4DDA-AF70-A2B1E7CF71F6}"/>
   </bookViews>
@@ -482,7 +482,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -624,6 +624,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3436,7 +3437,7 @@
         <v>40</v>
       </c>
       <c r="M11">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.35">
@@ -3462,7 +3463,7 @@
         <v>39</v>
       </c>
       <c r="M12">
-        <v>0.01</v>
+        <v>1E-3</v>
       </c>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.35">
@@ -3475,8 +3476,8 @@
       <c r="E13" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F13" s="20">
-        <v>8000</v>
+      <c r="F13" s="51">
+        <v>4000</v>
       </c>
       <c r="I13" s="20" t="s">
         <v>8</v>
@@ -3488,7 +3489,7 @@
         <v>41</v>
       </c>
       <c r="M13" s="20">
-        <v>8000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.35">
@@ -3504,7 +3505,7 @@
       </c>
       <c r="F16" s="22">
         <f>+(F12/F11)^(1/F13)</f>
-        <v>0.99942451937928012</v>
+        <v>0.99884936993650519</v>
       </c>
       <c r="I16" s="21" t="s">
         <v>41</v>
@@ -3518,7 +3519,7 @@
       </c>
       <c r="M16" s="22">
         <f>+(M12/M11)^(1/M13)</f>
-        <v>0.99962560356964758</v>
+        <v>0.99884936993650519</v>
       </c>
     </row>
     <row r="20" spans="4:13" x14ac:dyDescent="0.35">
@@ -3527,14 +3528,14 @@
       </c>
       <c r="F20">
         <f>+MAX($F$12,$F$11*$F$16^E20)</f>
-        <v>0.99942451937928012</v>
+        <v>0.99884936993650519</v>
       </c>
       <c r="L20">
         <v>1</v>
       </c>
       <c r="M20">
         <f>+MAX($M$12,$M$11*$M$16^L20)</f>
-        <v>0.19992512071392954</v>
+        <v>9.988493699365053E-2</v>
       </c>
     </row>
     <row r="21" spans="4:13" x14ac:dyDescent="0.35">
@@ -3543,14 +3544,14 @@
       </c>
       <c r="F21">
         <f t="shared" ref="F21:F30" si="0">+MAX($F$12,$F$11*$F$16^E21)</f>
-        <v>0.74989420933244089</v>
+        <v>0.56234132519035773</v>
       </c>
       <c r="L21">
         <v>500</v>
       </c>
       <c r="M21">
         <f t="shared" ref="M21:M30" si="1">+MAX($M$12,$M$11*$M$16^L21)</f>
-        <v>0.16585005540350253</v>
+        <v>5.6234132519035779E-2</v>
       </c>
     </row>
     <row r="22" spans="4:13" x14ac:dyDescent="0.35">
@@ -3559,14 +3560,14 @@
       </c>
       <c r="F22">
         <f t="shared" si="0"/>
-        <v>0.56234132519032654</v>
+        <v>0.3162277660168476</v>
       </c>
       <c r="L22">
         <v>1000</v>
       </c>
       <c r="M22">
         <f t="shared" si="1"/>
-        <v>0.13753120438672425</v>
+        <v>3.1622776601684763E-2</v>
       </c>
     </row>
     <row r="23" spans="4:13" x14ac:dyDescent="0.35">
@@ -3575,14 +3576,14 @@
       </c>
       <c r="F23">
         <f t="shared" si="0"/>
-        <v>0.42169650342855686</v>
+        <v>0.17782794100390042</v>
       </c>
       <c r="L23">
         <v>1500</v>
       </c>
       <c r="M23">
         <f t="shared" si="1"/>
-        <v>0.11404778933624325</v>
+        <v>1.7782794100390045E-2</v>
       </c>
     </row>
     <row r="24" spans="4:13" x14ac:dyDescent="0.35">
@@ -3591,14 +3592,14 @@
       </c>
       <c r="F24">
         <f t="shared" si="0"/>
-        <v>0.31622776601681257</v>
+        <v>0.1000000000000061</v>
       </c>
       <c r="L24">
         <v>2000</v>
       </c>
       <c r="M24">
         <f t="shared" si="1"/>
-        <v>9.4574160900314633E-2</v>
+        <v>1.0000000000000611E-2</v>
       </c>
     </row>
     <row r="25" spans="4:13" x14ac:dyDescent="0.35">
@@ -3607,14 +3608,14 @@
       </c>
       <c r="F25">
         <f t="shared" si="0"/>
-        <v>0.23713737056614176</v>
+        <v>5.6234132519039193E-2</v>
       </c>
       <c r="L25">
         <v>2500</v>
       </c>
       <c r="M25">
         <f t="shared" si="1"/>
-        <v>7.8425649125284713E-2</v>
+        <v>5.6234132519039194E-3</v>
       </c>
     </row>
     <row r="26" spans="4:13" x14ac:dyDescent="0.35">
@@ -3624,14 +3625,14 @@
       </c>
       <c r="F26">
         <f t="shared" si="0"/>
-        <v>0.17782794100387092</v>
+        <v>3.1622776601686692E-2</v>
       </c>
       <c r="L26">
         <v>3000</v>
       </c>
       <c r="M26">
         <f t="shared" si="1"/>
-        <v>6.5034491262420599E-2</v>
+        <v>3.1622776601686695E-3</v>
       </c>
     </row>
     <row r="27" spans="4:13" x14ac:dyDescent="0.35">
@@ -3641,14 +3642,14 @@
       </c>
       <c r="F27">
         <f t="shared" si="0"/>
-        <v>0.1333521432163137</v>
+        <v>1.7782794100391124E-2</v>
       </c>
       <c r="L27">
         <v>3500</v>
       </c>
       <c r="M27">
         <f t="shared" si="1"/>
-        <v>5.3929869895055285E-2</v>
+        <v>1.7782794100391125E-3</v>
       </c>
     </row>
     <row r="28" spans="4:13" x14ac:dyDescent="0.35">
@@ -3658,14 +3659,14 @@
       </c>
       <c r="F28">
         <f t="shared" si="0"/>
-        <v>9.9999999999983977E-2</v>
+        <v>1.000000000000122E-2</v>
       </c>
       <c r="L28">
         <v>4000</v>
       </c>
       <c r="M28">
         <f t="shared" si="1"/>
-        <v>4.4721359549993012E-2</v>
+        <v>1.0000000000001221E-3</v>
       </c>
     </row>
     <row r="29" spans="4:13" x14ac:dyDescent="0.35">
@@ -3675,14 +3676,14 @@
       </c>
       <c r="F29">
         <f t="shared" si="0"/>
-        <v>7.4989420933232062E-2</v>
+        <v>0.01</v>
       </c>
       <c r="L29">
         <v>4500</v>
       </c>
       <c r="M29">
         <f t="shared" si="1"/>
-        <v>3.7085199795431484E-2</v>
+        <v>1E-3</v>
       </c>
     </row>
     <row r="30" spans="4:13" x14ac:dyDescent="0.35">
@@ -3692,14 +3693,14 @@
       </c>
       <c r="F30">
         <f t="shared" si="0"/>
-        <v>5.6234132519023636E-2</v>
+        <v>0.01</v>
       </c>
       <c r="L30">
         <v>5000</v>
       </c>
       <c r="M30">
         <f t="shared" si="1"/>
-        <v>3.0752912203611361E-2</v>
+        <v>1E-3</v>
       </c>
     </row>
     <row r="31" spans="4:13" x14ac:dyDescent="0.35">
@@ -3709,14 +3710,14 @@
       </c>
       <c r="F31">
         <f t="shared" ref="F31:F37" si="2">+MAX($F$12,$F$11*$F$16^E31)</f>
-        <v>4.2169650342848926E-2</v>
+        <v>0.01</v>
       </c>
       <c r="L31">
         <v>5500</v>
       </c>
       <c r="M31">
         <f t="shared" ref="M31:M36" si="3">+MAX($M$12,$M$11*$M$16^L31)</f>
-        <v>2.5501860963939967E-2</v>
+        <v>1E-3</v>
       </c>
     </row>
     <row r="32" spans="4:13" x14ac:dyDescent="0.35">
@@ -3725,14 +3726,14 @@
       </c>
       <c r="F32">
         <f t="shared" si="2"/>
-        <v>3.1622776601676186E-2</v>
+        <v>0.01</v>
       </c>
       <c r="L32">
         <v>6000</v>
       </c>
       <c r="M32">
         <f t="shared" si="3"/>
-        <v>2.1147425268809306E-2</v>
+        <v>1E-3</v>
       </c>
     </row>
     <row r="33" spans="5:13" x14ac:dyDescent="0.35">
@@ -3741,14 +3742,14 @@
       </c>
       <c r="F33">
         <f t="shared" si="2"/>
-        <v>2.3713737056610371E-2</v>
+        <v>0.01</v>
       </c>
       <c r="L33">
         <v>6500</v>
       </c>
       <c r="M33">
         <f t="shared" si="3"/>
-        <v>1.7536508262367263E-2</v>
+        <v>1E-3</v>
       </c>
     </row>
     <row r="34" spans="5:13" x14ac:dyDescent="0.35">
@@ -3757,14 +3758,14 @@
       </c>
       <c r="F34">
         <f t="shared" si="2"/>
-        <v>1.7782794100384237E-2</v>
+        <v>0.01</v>
       </c>
       <c r="L34">
         <v>7000</v>
       </c>
       <c r="M34">
         <f t="shared" si="3"/>
-        <v>1.4542154334487953E-2</v>
+        <v>1E-3</v>
       </c>
     </row>
     <row r="35" spans="5:13" x14ac:dyDescent="0.35">
@@ -3773,14 +3774,14 @@
       </c>
       <c r="F35">
         <f t="shared" si="2"/>
-        <v>1.3335214321629228E-2</v>
+        <v>0.01</v>
       </c>
       <c r="L35">
         <v>7500</v>
       </c>
       <c r="M35">
         <f t="shared" si="3"/>
-        <v>1.2059085510305555E-2</v>
+        <v>1E-3</v>
       </c>
     </row>
     <row r="36" spans="5:13" x14ac:dyDescent="0.35">
@@ -3796,7 +3797,7 @@
       </c>
       <c r="M36">
         <f t="shared" si="3"/>
-        <v>0.01</v>
+        <v>1E-3</v>
       </c>
     </row>
     <row r="37" spans="5:13" x14ac:dyDescent="0.35">
@@ -3812,7 +3813,7 @@
       </c>
       <c r="M37">
         <f t="shared" ref="M37" si="4">+MAX($M$12,$M$11*$M$16^L37)</f>
-        <v>0.01</v>
+        <v>1E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>